<commit_message>
update image and list
</commit_message>
<xml_diff>
--- a/product/product list-event price.xlsx
+++ b/product/product list-event price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\meowmeow_sandbox\product\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67E98EB5-C9A2-4B5F-9819-2FC3A854209D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A83F24-DCF3-4D2A-AD89-0832BFBFF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2757FED6-37E3-4677-8046-0F44B021E7C6}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
   <si>
     <t>Brand</t>
   </si>
@@ -94,12 +94,6 @@
   </si>
   <si>
     <t>The sphinx of Giza</t>
-  </si>
-  <si>
-    <t>011</t>
-  </si>
-  <si>
-    <t>The sphinx of Greeze</t>
   </si>
   <si>
     <t>012</t>
@@ -284,7 +278,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -341,9 +335,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -681,7 +672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1F0F27A-D109-48B1-987B-4F9F9BC6EC42}">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.6328125" customWidth="1"/>
@@ -706,13 +697,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.4">
@@ -736,7 +727,7 @@
         <v>140</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
@@ -756,11 +747,11 @@
         <v>650</v>
       </c>
       <c r="F3" s="12">
-        <f t="shared" ref="F3:F24" si="0">D3-E3</f>
+        <f t="shared" ref="F3:F20" si="0">D3-E3</f>
         <v>140</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -894,63 +885,63 @@
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="14">
-        <v>990</v>
+      <c r="D10" s="13">
+        <v>1590</v>
       </c>
       <c r="E10" s="12">
-        <v>890</v>
+        <v>1290</v>
       </c>
       <c r="F10" s="12">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="13">
-        <v>1590</v>
+      <c r="D11" s="14">
+        <v>1990</v>
       </c>
       <c r="E11" s="12">
-        <v>1290</v>
+        <v>1490</v>
       </c>
       <c r="F11" s="12">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="14">
-        <v>1990</v>
+      <c r="D12" s="13">
+        <v>790</v>
       </c>
       <c r="E12" s="12">
-        <v>1490</v>
+        <v>590</v>
       </c>
       <c r="F12" s="12">
         <f t="shared" si="0"/>
-        <v>500</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
@@ -964,14 +955,14 @@
         <v>27</v>
       </c>
       <c r="D13" s="13">
-        <v>790</v>
+        <v>1690</v>
       </c>
       <c r="E13" s="12">
-        <v>590</v>
+        <v>1390</v>
       </c>
       <c r="F13" s="12">
         <f t="shared" si="0"/>
-        <v>200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
@@ -982,49 +973,49 @@
         <v>28</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="D14" s="13">
         <v>1690</v>
       </c>
       <c r="E14" s="12">
-        <v>1390</v>
+        <v>1490</v>
       </c>
       <c r="F14" s="12">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="13">
-        <v>1690</v>
-      </c>
-      <c r="E15" s="12">
-        <v>1490</v>
-      </c>
-      <c r="F15" s="12">
-        <f t="shared" si="0"/>
-        <v>200</v>
+      <c r="C15" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="15">
+        <v>590</v>
+      </c>
+      <c r="E15" s="16">
+        <v>450</v>
+      </c>
+      <c r="F15" s="16">
+        <f t="shared" si="0"/>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>32</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>47</v>
       </c>
       <c r="D16" s="15">
         <v>590</v>
@@ -1039,34 +1030,34 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="10" t="s">
-        <v>34</v>
+      <c r="C17" s="21" t="s">
+        <v>46</v>
       </c>
       <c r="D17" s="15">
-        <v>590</v>
+        <v>890</v>
       </c>
       <c r="E17" s="16">
-        <v>450</v>
+        <v>650</v>
       </c>
       <c r="F17" s="16">
         <f t="shared" si="0"/>
-        <v>140</v>
+        <v>240</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D18" s="15">
         <v>890</v>
@@ -1080,24 +1071,24 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="15">
-        <v>890</v>
-      </c>
-      <c r="E19" s="16">
-        <v>650</v>
-      </c>
-      <c r="F19" s="16">
-        <f t="shared" si="0"/>
-        <v>240</v>
+      <c r="A19" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="12">
+        <v>100</v>
+      </c>
+      <c r="E19" s="12">
+        <v>100</v>
+      </c>
+      <c r="F19" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
@@ -1105,10 +1096,10 @@
         <v>3</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" s="12">
         <v>100</v>
@@ -1122,25 +1113,11 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="12">
-        <v>100</v>
-      </c>
-      <c r="E21" s="12">
-        <v>100</v>
-      </c>
-      <c r="F21" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="A21" s="3"/>
+      <c r="B21" s="7"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
@@ -1156,13 +1133,6 @@
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" s="3"/>
-      <c r="B24" s="7"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update delivery cost and change promo
</commit_message>
<xml_diff>
--- a/product/product list-event price.xlsx
+++ b/product/product list-event price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\meowmeow_sandbox\product\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A83F24-DCF3-4D2A-AD89-0832BFBFF0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF52C4E8-F8D0-4198-AE37-5F2EB17EBF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2757FED6-37E3-4677-8046-0F44B021E7C6}"/>
   </bookViews>
@@ -34,10 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
-  <si>
-    <t>Brand</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>SKU</t>
   </si>
@@ -45,9 +42,6 @@
     <t>Description</t>
   </si>
   <si>
-    <t>The Meowseum</t>
-  </si>
-  <si>
     <t>002A</t>
   </si>
   <si>
@@ -121,9 +115,6 @@
   </si>
   <si>
     <t>016</t>
-  </si>
-  <si>
-    <t>Modern Friends</t>
   </si>
   <si>
     <t>017</t>
@@ -163,12 +154,6 @@
     <t>Promotion Pet Expo</t>
   </si>
   <si>
-    <t>ซื้อครบ 2,000 บาท (Meowsuem+Modern Friends) ฟรี ผ้าพันคอ Limited Edition Meowsuem มูลค่า 390 บาท</t>
-  </si>
-  <si>
-    <t>Promotion Price (event price)</t>
-  </si>
-  <si>
     <t>Royal Haus of Meow</t>
   </si>
   <si>
@@ -179,6 +164,15 @@
   </si>
   <si>
     <t>Ribbon Bow</t>
+  </si>
+  <si>
+    <t>Promotion Price</t>
+  </si>
+  <si>
+    <t>Delivery Fee</t>
+  </si>
+  <si>
+    <t>ซื้อครบ 1200 บาท (Meowsuem+Modern Friends) ฟรี Sticker Meowsuem 1 ชิ้น(sku:021 or 022) มูลค่า 100 บาท</t>
   </si>
 </sst>
 </file>
@@ -242,12 +236,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -261,6 +249,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -283,9 +277,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -301,13 +292,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -322,20 +313,21 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -675,13 +667,13 @@
   <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.6328125" customWidth="1"/>
-    <col min="2" max="2" width="5.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.90625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.08984375" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.54296875" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="89.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.08984375" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="92.6328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.90625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -690,448 +682,442 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>38</v>
+      <c r="E1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>5</v>
+      <c r="C2" s="10">
+        <v>790</v>
       </c>
       <c r="D2" s="11">
-        <v>790</v>
-      </c>
-      <c r="E2" s="12">
         <v>650</v>
       </c>
-      <c r="F2" s="12">
-        <f>D2-E2</f>
+      <c r="E2" s="11">
+        <f>C2-D2</f>
         <v>140</v>
       </c>
-      <c r="H2" s="19" t="s">
-        <v>41</v>
+      <c r="F2" s="11">
+        <v>120</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="C3" s="10">
+        <v>790</v>
       </c>
       <c r="D3" s="11">
-        <v>790</v>
-      </c>
-      <c r="E3" s="12">
         <v>650</v>
       </c>
-      <c r="F3" s="12">
-        <f t="shared" ref="F3:F20" si="0">D3-E3</f>
+      <c r="E3" s="11">
+        <f t="shared" ref="E3:E20" si="0">C3-D3</f>
         <v>140</v>
       </c>
-      <c r="H3" s="18" t="s">
-        <v>42</v>
+      <c r="F3" s="11">
+        <v>120</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C4" s="10">
+        <v>890</v>
       </c>
       <c r="D4" s="11">
-        <v>890</v>
-      </c>
-      <c r="E4" s="12">
         <v>790</v>
       </c>
-      <c r="F4" s="12">
+      <c r="E4" s="11">
         <f t="shared" si="0"/>
         <v>100</v>
+      </c>
+      <c r="F4" s="11">
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
+      </c>
+      <c r="C5" s="10">
+        <v>490</v>
       </c>
       <c r="D5" s="11">
-        <v>490</v>
-      </c>
-      <c r="E5" s="12">
         <v>450</v>
       </c>
-      <c r="F5" s="12">
+      <c r="E5" s="11">
         <f t="shared" si="0"/>
         <v>40</v>
+      </c>
+      <c r="F5" s="11">
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
+      </c>
+      <c r="C6" s="10">
+        <v>2590</v>
       </c>
       <c r="D6" s="11">
-        <v>2590</v>
-      </c>
-      <c r="E6" s="12">
         <v>2190</v>
       </c>
-      <c r="F6" s="12">
+      <c r="E6" s="11">
         <f t="shared" si="0"/>
         <v>400</v>
+      </c>
+      <c r="F6" s="11">
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="13">
+        <v>13</v>
+      </c>
+      <c r="C7" s="12">
         <v>990</v>
       </c>
-      <c r="E7" s="12">
+      <c r="D7" s="11">
         <v>790</v>
       </c>
-      <c r="F7" s="12">
+      <c r="E7" s="11">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
-      <c r="L7" s="17"/>
+      <c r="F7" s="11">
+        <v>120</v>
+      </c>
+      <c r="L7" s="16"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="13">
+        <v>15</v>
+      </c>
+      <c r="C8" s="12">
         <v>1190</v>
       </c>
-      <c r="E8" s="12">
+      <c r="D8" s="11">
         <v>990</v>
       </c>
-      <c r="F8" s="12">
-        <f t="shared" si="0"/>
+      <c r="E8" s="11">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+      <c r="F8" s="11">
         <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="13">
+        <v>17</v>
+      </c>
+      <c r="C9" s="12">
         <v>790</v>
       </c>
-      <c r="E9" s="12">
+      <c r="D9" s="11">
         <v>690</v>
       </c>
-      <c r="F9" s="12">
+      <c r="E9" s="11">
         <f t="shared" si="0"/>
         <v>100</v>
+      </c>
+      <c r="F9" s="11">
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="12">
+        <v>1590</v>
+      </c>
+      <c r="D10" s="11">
+        <v>1290</v>
+      </c>
+      <c r="E10" s="11">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="F10" s="11">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="B11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="13">
-        <v>1590</v>
-      </c>
-      <c r="E10" s="12">
-        <v>1290</v>
-      </c>
-      <c r="F10" s="12">
-        <f t="shared" si="0"/>
-        <v>300</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="14">
+      <c r="C11" s="13">
         <v>1990</v>
       </c>
-      <c r="E11" s="12">
+      <c r="D11" s="11">
         <v>1490</v>
       </c>
-      <c r="F11" s="12">
+      <c r="E11" s="11">
         <f t="shared" si="0"/>
         <v>500</v>
+      </c>
+      <c r="F11" s="11">
+        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="13">
+        <v>23</v>
+      </c>
+      <c r="C12" s="12">
         <v>790</v>
       </c>
-      <c r="E12" s="12">
+      <c r="D12" s="11">
         <v>590</v>
       </c>
-      <c r="F12" s="12">
+      <c r="E12" s="11">
         <f t="shared" si="0"/>
         <v>200</v>
+      </c>
+      <c r="F12" s="11">
+        <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="13">
+        <v>25</v>
+      </c>
+      <c r="C13" s="12">
         <v>1690</v>
       </c>
-      <c r="E13" s="12">
+      <c r="D13" s="11">
         <v>1390</v>
       </c>
-      <c r="F13" s="12">
+      <c r="E13" s="11">
         <f t="shared" si="0"/>
         <v>300</v>
+      </c>
+      <c r="F13" s="11">
+        <v>200</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="13">
+        <v>39</v>
+      </c>
+      <c r="C14" s="12">
         <v>1690</v>
       </c>
-      <c r="E14" s="12">
+      <c r="D14" s="11">
         <v>1490</v>
       </c>
-      <c r="F14" s="12">
+      <c r="E14" s="11">
         <f t="shared" si="0"/>
         <v>200</v>
       </c>
+      <c r="F14" s="11">
+        <v>200</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A15" s="8" t="s">
-        <v>29</v>
+      <c r="A15" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>45</v>
+        <v>40</v>
+      </c>
+      <c r="C15" s="14">
+        <v>590</v>
       </c>
       <c r="D15" s="15">
-        <v>590</v>
-      </c>
-      <c r="E15" s="16">
         <v>450</v>
       </c>
-      <c r="F15" s="16">
+      <c r="E15" s="15">
         <f t="shared" si="0"/>
         <v>140</v>
+      </c>
+      <c r="F15" s="11">
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>32</v>
+      <c r="C16" s="14">
+        <v>590</v>
       </c>
       <c r="D16" s="15">
-        <v>590</v>
-      </c>
-      <c r="E16" s="16">
         <v>450</v>
       </c>
-      <c r="F16" s="16">
+      <c r="E16" s="15">
         <f t="shared" si="0"/>
         <v>140</v>
       </c>
+      <c r="F16" s="20"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>46</v>
+        <v>30</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="14">
+        <v>890</v>
       </c>
       <c r="D17" s="15">
-        <v>890</v>
-      </c>
-      <c r="E17" s="16">
         <v>650</v>
       </c>
-      <c r="F17" s="16">
+      <c r="E17" s="15">
         <f t="shared" si="0"/>
         <v>240</v>
+      </c>
+      <c r="F17" s="11">
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>47</v>
+        <v>31</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="14">
+        <v>890</v>
       </c>
       <c r="D18" s="15">
-        <v>890</v>
-      </c>
-      <c r="E18" s="16">
         <v>650</v>
       </c>
-      <c r="F18" s="16">
+      <c r="E18" s="15">
         <f t="shared" si="0"/>
         <v>240</v>
       </c>
+      <c r="F18" s="11">
+        <v>50</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="12">
+      <c r="A19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="11">
         <v>100</v>
       </c>
-      <c r="E19" s="12">
+      <c r="D19" s="11">
         <v>100</v>
       </c>
-      <c r="F19" s="12">
+      <c r="E19" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="F19" s="21"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" s="12">
+        <v>33</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="11">
         <v>100</v>
       </c>
-      <c r="E20" s="12">
+      <c r="D20" s="11">
         <v>100</v>
       </c>
-      <c r="F20" s="12">
+      <c r="E20" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="F20" s="21"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="3"/>
-      <c r="B21" s="7"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
+      <c r="A21" s="2"/>
+      <c r="B21" s="6"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="3"/>
-      <c r="B22" s="7"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
+      <c r="A22" s="2"/>
+      <c r="B22" s="6"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="3"/>
-      <c r="B23" s="7"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
+      <c r="A23" s="2"/>
+      <c r="B23" s="6"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>